<commit_message>
Add Revolut to payment matrix
</commit_message>
<xml_diff>
--- a/cross_border_ecommerce_payment_matrix.xlsx
+++ b/cross_border_ecommerce_payment_matrix.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R33283fb888f04f7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Country Matrix" sheetId="2" r:id="R6bd6f3f891bb47fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider Matrix" sheetId="3" r:id="R01a424484ce94ac2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payment Methods" sheetId="4" r:id="R1056b1e2200b45f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seller Stack" sheetId="5" r:id="Rbeee9341d0014300"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R02cd5289f4e64800"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7a501fa28c9d4661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Country Matrix" sheetId="2" r:id="R652912ba4ed94eed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider Matrix" sheetId="3" r:id="Ra4fbd091054a4761"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payment Methods" sheetId="4" r:id="Rd00937797fc049ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seller Stack" sheetId="5" r:id="R670eb4a85ccb4461"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R1e18908719674618"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -590,7 +590,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R75263b2ffbba46bf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rba7b55435dd74785"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -865,7 +865,7 @@
       </x:c>
       <x:c r="B6" s="53" t="n">
         <x:f>COUNTA('Provider Matrix'!A2:A80)</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C6" s="53"/>
       <x:c r="D6" s="53" t="str">
@@ -895,7 +895,7 @@
       </x:c>
       <x:c r="B7" s="53" t="n">
         <x:f>COUNTA('Payment Methods'!A2:A80)</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C7" s="53"/>
       <x:c r="D7" s="53" t="str">
@@ -997,11 +997,11 @@
       </x:c>
       <x:c r="G10" s="53" t="str">
         <x:f>IF(D10="","",INDEX('Country Matrix'!$I$2:$I$50,MATCH(D10,'Country Matrix'!$A$2:$A$50,0)))</x:f>
-        <x:v>Stripe/Shopify + PayPal + Klarna/Clearpay</x:v>
+        <x:v>Stripe/Shopify + PayPal + Klarna/Clearpay; Revolut as FX/merchant add-on</x:v>
       </x:c>
       <x:c r="H10" s="54" t="str">
         <x:f>IF(D10="","",INDEX('Country Matrix'!$L$2:$L$50,MATCH(D10,'Country Matrix'!$A$2:$A$50,0)))</x:f>
-        <x:v>Test after US if product has high AOV and clear value prop.</x:v>
+        <x:v>Test after US; evaluate Revolut Business if UK entity/settlement matters.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1022,7 +1022,7 @@
       </x:c>
       <x:c r="G11" s="53" t="str">
         <x:f>IF(D11="","",INDEX('Country Matrix'!$I$2:$I$50,MATCH(D11,'Country Matrix'!$A$2:$A$50,0)))</x:f>
-        <x:v>Shopify/Stripe + PayPal + Afterpay</x:v>
+        <x:v>Shopify/Stripe + PayPal + Afterpay; evaluate Revolut for AU entity</x:v>
       </x:c>
       <x:c r="H11" s="54" t="str">
         <x:f>IF(D11="","",INDEX('Country Matrix'!$L$2:$L$50,MATCH(D11,'Country Matrix'!$A$2:$A$50,0)))</x:f>
@@ -1047,7 +1047,7 @@
       </x:c>
       <x:c r="G12" s="53" t="str">
         <x:f>IF(D12="","",INDEX('Country Matrix'!$I$2:$I$50,MATCH(D12,'Country Matrix'!$A$2:$A$50,0)))</x:f>
-        <x:v>Stripe/Shopify + PayPal + Bizum/SEPA/Klarna where available</x:v>
+        <x:v>Stripe/Shopify + PayPal + Bizum/SEPA/Klarna; Revolut as EU FX/checkout add-on</x:v>
       </x:c>
       <x:c r="H12" s="54" t="str">
         <x:f>IF(D12="","",INDEX('Country Matrix'!$L$2:$L$50,MATCH(D12,'Country Matrix'!$A$2:$A$50,0)))</x:f>
@@ -1130,7 +1130,7 @@
         <x:v>Example</x:v>
       </x:c>
       <x:c r="E17" s="53" t="str">
-        <x:v>Airwallex, Payoneer, WorldFirst, PingPong, LianLian, Wise</x:v>
+        <x:v>Airwallex, Revolut, Payoneer, WorldFirst, PingPong, LianLian, Wise</x:v>
       </x:c>
       <x:c r="F17" s="53" t="str"/>
       <x:c r="G17" s="53" t="str"/>
@@ -1158,7 +1158,7 @@
     <x:mergeCell ref="A14:H14"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c95374a57a14e38"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10d2b448b8a443b6"/>
 </x:worksheet>
 </file>
 
@@ -1468,16 +1468,16 @@
         <x:v>High ecommerce maturity and strong DTC habit.</x:v>
       </x:c>
       <x:c r="F7" s="53" t="str">
-        <x:v>Cards, PayPal, Apple Pay, Google Pay, Klarna/Clearpay, Open Banking</x:v>
+        <x:v>Cards, PayPal, Apple Pay, Google Pay, Revolut Pay, Klarna/Clearpay, Open Banking</x:v>
       </x:c>
       <x:c r="G7" s="53" t="str">
-        <x:v>Stripe; Shopify Payments; PayPal; Adyen; Checkout.com; Klarna</x:v>
+        <x:v>Stripe; Shopify Payments; PayPal; Adyen; Checkout.com; Klarna; Revolut Business</x:v>
       </x:c>
       <x:c r="H7" s="53" t="str">
-        <x:v>Airwallex; Wise Business; Payoneer</x:v>
+        <x:v>Airwallex; Revolut Business; Wise Business; Payoneer</x:v>
       </x:c>
       <x:c r="I7" s="53" t="str">
-        <x:v>Stripe/Shopify + PayPal + Klarna/Clearpay</x:v>
+        <x:v>Stripe/Shopify + PayPal + Klarna/Clearpay; Revolut as FX/merchant add-on</x:v>
       </x:c>
       <x:c r="J7" s="53" t="str">
         <x:v>VAT, product safety, return expectations.</x:v>
@@ -1486,10 +1486,10 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L7" s="53" t="str">
-        <x:v>Test after US if product has high AOV and clear value prop.</x:v>
+        <x:v>Test after US; evaluate Revolut Business if UK entity/settlement matters.</x:v>
       </x:c>
       <x:c r="M7" s="53" t="str">
-        <x:v>S01; S02; S03; S04</x:v>
+        <x:v>S01; S02; S03; S04; S31; S32; S33; S34</x:v>
       </x:c>
       <x:c r="N7" s="54" t="n">
         <x:f>COUNTIF($C$2:$C$15,"&gt;"&amp;C7)+COUNTIF($C$2:C7,C7)</x:f>
@@ -1516,13 +1516,13 @@
         <x:v>Cards, PayPal, Apple Pay, Google Pay, Afterpay, PayTo/PayID</x:v>
       </x:c>
       <x:c r="G8" s="53" t="str">
-        <x:v>Stripe; Shopify Payments; PayPal; Adyen; Afterpay</x:v>
+        <x:v>Stripe; Shopify Payments; PayPal; Adyen; Afterpay; Revolut Business (AU)</x:v>
       </x:c>
       <x:c r="H8" s="53" t="str">
-        <x:v>Airwallex; Wise Business; Payoneer</x:v>
+        <x:v>Airwallex; Revolut Business; Wise Business; Payoneer</x:v>
       </x:c>
       <x:c r="I8" s="53" t="str">
-        <x:v>Shopify/Stripe + PayPal + Afterpay</x:v>
+        <x:v>Shopify/Stripe + PayPal + Afterpay; evaluate Revolut for AU entity</x:v>
       </x:c>
       <x:c r="J8" s="53" t="str">
         <x:v>Freight distance, GST, returns.</x:v>
@@ -1534,7 +1534,7 @@
         <x:v>Use only for light, high-margin products.</x:v>
       </x:c>
       <x:c r="M8" s="53" t="str">
-        <x:v>S01; S02; S03; S21</x:v>
+        <x:v>S01; S02; S03; S21; S31; S32; S34</x:v>
       </x:c>
       <x:c r="N8" s="54" t="n">
         <x:f>COUNTIF($C$2:$C$15,"&gt;"&amp;C8)+COUNTIF($C$2:C8,C8)</x:f>
@@ -1558,16 +1558,16 @@
         <x:v>Spanish-language market with EU purchasing power; compliance is heavier.</x:v>
       </x:c>
       <x:c r="F9" s="53" t="str">
-        <x:v>Cards/debit, PayPal, Apple Pay, Google Pay, Bizum, SEPA, Klarna</x:v>
+        <x:v>Cards/debit, PayPal, Apple Pay, Google Pay, Revolut Pay, Bizum, SEPA, Klarna</x:v>
       </x:c>
       <x:c r="G9" s="53" t="str">
-        <x:v>Stripe; Shopify Payments; PayPal; Adyen; Klarna; local PSPs</x:v>
+        <x:v>Stripe; Shopify Payments; PayPal; Adyen; Klarna; Revolut Business; local PSPs</x:v>
       </x:c>
       <x:c r="H9" s="53" t="str">
-        <x:v>Airwallex; Wise Business; Payoneer</x:v>
+        <x:v>Airwallex; Revolut Business; Wise Business; Payoneer</x:v>
       </x:c>
       <x:c r="I9" s="53" t="str">
-        <x:v>Stripe/Shopify + PayPal + Bizum/SEPA/Klarna where available</x:v>
+        <x:v>Stripe/Shopify + PayPal + Bizum/SEPA/Klarna; Revolut as EU FX/checkout add-on</x:v>
       </x:c>
       <x:c r="J9" s="53" t="str">
         <x:v>VAT/IOSS, GPSR, EU returns, Spanish customer support.</x:v>
@@ -1579,7 +1579,7 @@
         <x:v>Prepare EU compliance checklist before paid ads.</x:v>
       </x:c>
       <x:c r="M9" s="53" t="str">
-        <x:v>S01; S02; S03; S04; S26; S27</x:v>
+        <x:v>S01; S02; S03; S04; S26; S27; S31; S32; S33; S34</x:v>
       </x:c>
       <x:c r="N9" s="54" t="n">
         <x:f>COUNTIF($C$2:$C$15,"&gt;"&amp;C9)+COUNTIF($C$2:C9,C9)</x:f>
@@ -1648,16 +1648,16 @@
         <x:v>Large EU ecommerce market with distinctive trust and payment preferences.</x:v>
       </x:c>
       <x:c r="F11" s="53" t="str">
-        <x:v>PayPal, invoice/BNPL, SEPA, cards, Klarna</x:v>
+        <x:v>PayPal, invoice/BNPL, SEPA, cards, Klarna, Revolut Pay</x:v>
       </x:c>
       <x:c r="G11" s="53" t="str">
-        <x:v>Adyen; Stripe; PayPal; Klarna; Shopify Payments</x:v>
+        <x:v>Adyen; Stripe; PayPal; Klarna; Shopify Payments; Revolut Business</x:v>
       </x:c>
       <x:c r="H11" s="53" t="str">
-        <x:v>Airwallex; Wise Business; Payoneer</x:v>
+        <x:v>Airwallex; Revolut Business; Wise Business; Payoneer</x:v>
       </x:c>
       <x:c r="I11" s="53" t="str">
-        <x:v>PayPal + cards + SEPA/Klarna</x:v>
+        <x:v>PayPal + cards + SEPA/Klarna; Revolut for EU account/payment add-on</x:v>
       </x:c>
       <x:c r="J11" s="53" t="str">
         <x:v>German language, return expectations, EU compliance.</x:v>
@@ -1669,7 +1669,7 @@
         <x:v>Enter after EU compliance and support are ready.</x:v>
       </x:c>
       <x:c r="M11" s="53" t="str">
-        <x:v>S01; S02; S03; S04; S26; S27</x:v>
+        <x:v>S01; S02; S03; S04; S26; S27; S31; S32; S34</x:v>
       </x:c>
       <x:c r="N11" s="54" t="n">
         <x:f>COUNTIF($C$2:$C$15,"&gt;"&amp;C11)+COUNTIF($C$2:C11,C11)</x:f>
@@ -2214,139 +2214,162 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="52" t="str">
-        <x:v>Airwallex</x:v>
+        <x:v>Revolut Business / Revolut Pay / Merchant Account</x:v>
       </x:c>
       <x:c r="B15" s="53" t="str">
-        <x:v>Seller settlement / FX / global accounts</x:v>
+        <x:v>Seller settlement + checkout add-on</x:v>
       </x:c>
       <x:c r="C15" s="53" t="str">
-        <x:v>Cross-border DTC and suppliers</x:v>
+        <x:v>UK/EU/Spain/Germany/Australia/Singapore; sellers with supported entity</x:v>
       </x:c>
       <x:c r="D15" s="53" t="str">
-        <x:v>Multi-currency accounts, FX, cards, payouts</x:v>
+        <x:v>Multi-currency accounts, FX, merchant account, Revolut Pay, payment gateway/plugins</x:v>
       </x:c>
       <x:c r="E15" s="53" t="str">
-        <x:v>Use early for USD/EUR/GBP receipts and supplier payments</x:v>
+        <x:v>Use when a UK/EU/AU entity wants FX, settlement, and checkout add-on in one account</x:v>
       </x:c>
       <x:c r="F15" s="53" t="str">
-        <x:v>KYC and compliance documents needed.</x:v>
+        <x:v>Merchant account countries are limited; not a Mexico/Brazil/Argentina local-payment answer; avoid using as sole PSP before testing.</x:v>
       </x:c>
       <x:c r="G15" s="54" t="str">
-        <x:v>S13</x:v>
+        <x:v>S31; S32; S33; S34</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="52" t="str">
-        <x:v>Payoneer</x:v>
+        <x:v>Airwallex</x:v>
       </x:c>
       <x:c r="B16" s="53" t="str">
-        <x:v>Marketplace payout / seller account</x:v>
+        <x:v>Seller settlement / FX / global accounts</x:v>
       </x:c>
       <x:c r="C16" s="53" t="str">
-        <x:v>Amazon, Walmart, eBay, marketplace sellers</x:v>
+        <x:v>Cross-border DTC and suppliers</x:v>
       </x:c>
       <x:c r="D16" s="53" t="str">
-        <x:v>Platform payouts, withdrawals, supplier payments</x:v>
+        <x:v>Multi-currency accounts, FX, cards, payouts</x:v>
       </x:c>
       <x:c r="E16" s="53" t="str">
-        <x:v>When selling through marketplaces</x:v>
+        <x:v>Use early for USD/EUR/GBP receipts and supplier payments</x:v>
       </x:c>
       <x:c r="F16" s="53" t="str">
-        <x:v>Account holds and platform binding rules.</x:v>
+        <x:v>KYC and compliance documents needed.</x:v>
       </x:c>
       <x:c r="G16" s="54" t="str">
-        <x:v>S14</x:v>
+        <x:v>S13</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="52" t="str">
-        <x:v>WorldFirst</x:v>
+        <x:v>Payoneer</x:v>
       </x:c>
       <x:c r="B17" s="53" t="str">
-        <x:v>Marketplace payout + supplier payments</x:v>
+        <x:v>Marketplace payout / seller account</x:v>
       </x:c>
       <x:c r="C17" s="53" t="str">
-        <x:v>Amazon/eBay/Shopee/Lazada/1688 related workflows</x:v>
+        <x:v>Amazon, Walmart, eBay, marketplace sellers</x:v>
       </x:c>
       <x:c r="D17" s="53" t="str">
-        <x:v>Multi-currency collection and supplier payments</x:v>
+        <x:v>Platform payouts, withdrawals, supplier payments</x:v>
       </x:c>
       <x:c r="E17" s="53" t="str">
-        <x:v>When China sourcing and marketplace sales combine</x:v>
+        <x:v>When selling through marketplaces</x:v>
       </x:c>
       <x:c r="F17" s="53" t="str">
-        <x:v>Coverage varies by country/platform.</x:v>
+        <x:v>Account holds and platform binding rules.</x:v>
       </x:c>
       <x:c r="G17" s="54" t="str">
-        <x:v>S15</x:v>
+        <x:v>S14</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="52" t="str">
-        <x:v>PingPong</x:v>
+        <x:v>WorldFirst</x:v>
       </x:c>
       <x:c r="B18" s="53" t="str">
-        <x:v>Marketplace/platform collection</x:v>
+        <x:v>Marketplace payout + supplier payments</x:v>
       </x:c>
       <x:c r="C18" s="53" t="str">
-        <x:v>Cross-border sellers and platforms</x:v>
+        <x:v>Amazon/eBay/Shopee/Lazada/1688 related workflows</x:v>
       </x:c>
       <x:c r="D18" s="53" t="str">
-        <x:v>Collection, FX, supplier payments</x:v>
+        <x:v>Multi-currency collection and supplier payments</x:v>
       </x:c>
       <x:c r="E18" s="53" t="str">
-        <x:v>Use as primary or backup seller account</x:v>
+        <x:v>When China sourcing and marketplace sales combine</x:v>
       </x:c>
       <x:c r="F18" s="53" t="str">
-        <x:v>Keep documentation and backup accounts.</x:v>
+        <x:v>Coverage varies by country/platform.</x:v>
       </x:c>
       <x:c r="G18" s="54" t="str">
-        <x:v>S16</x:v>
+        <x:v>S15</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="52" t="str">
+        <x:v>PingPong</x:v>
+      </x:c>
+      <x:c r="B19" s="53" t="str">
+        <x:v>Marketplace/platform collection</x:v>
+      </x:c>
+      <x:c r="C19" s="53" t="str">
+        <x:v>Cross-border sellers and platforms</x:v>
+      </x:c>
+      <x:c r="D19" s="53" t="str">
+        <x:v>Collection, FX, supplier payments</x:v>
+      </x:c>
+      <x:c r="E19" s="53" t="str">
+        <x:v>Use as primary or backup seller account</x:v>
+      </x:c>
+      <x:c r="F19" s="53" t="str">
+        <x:v>Keep documentation and backup accounts.</x:v>
+      </x:c>
+      <x:c r="G19" s="54" t="str">
+        <x:v>S16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="52" t="str">
         <x:v>LianLian Global</x:v>
       </x:c>
-      <x:c r="B19" s="53" t="str">
+      <x:c r="B20" s="53" t="str">
         <x:v>Cross-border collection/payment</x:v>
       </x:c>
-      <x:c r="C19" s="53" t="str">
+      <x:c r="C20" s="53" t="str">
         <x:v>China-based sellers and global merchants</x:v>
       </x:c>
-      <x:c r="D19" s="53" t="str">
+      <x:c r="D20" s="53" t="str">
         <x:v>Global collection, payout, merchant services</x:v>
       </x:c>
-      <x:c r="E19" s="53" t="str">
+      <x:c r="E20" s="53" t="str">
         <x:v>Useful China-seller payment stack option</x:v>
       </x:c>
-      <x:c r="F19" s="53" t="str">
+      <x:c r="F20" s="53" t="str">
         <x:v>Confirm country and platform support.</x:v>
       </x:c>
-      <x:c r="G19" s="54" t="str">
+      <x:c r="G20" s="54" t="str">
         <x:v>S17</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="63" t="str">
+    <x:row r="21">
+      <x:c r="A21" s="63" t="str">
         <x:v>Wise Business</x:v>
       </x:c>
-      <x:c r="B20" s="64" t="str">
+      <x:c r="B21" s="64" t="str">
         <x:v>Multi-currency account / transfer</x:v>
       </x:c>
-      <x:c r="C20" s="64" t="str">
+      <x:c r="C21" s="64" t="str">
         <x:v>US/EU/UK/AU and supplier payments</x:v>
       </x:c>
-      <x:c r="D20" s="64" t="str">
+      <x:c r="D21" s="64" t="str">
         <x:v>Low-friction FX and international transfers</x:v>
       </x:c>
-      <x:c r="E20" s="64" t="str">
+      <x:c r="E21" s="64" t="str">
         <x:v>Use as auxiliary FX/transfer account</x:v>
       </x:c>
-      <x:c r="F20" s="64" t="str">
+      <x:c r="F21" s="64" t="str">
         <x:v>Not a full buyer checkout PSP.</x:v>
       </x:c>
-      <x:c r="G20" s="65" t="str">
+      <x:c r="G21" s="65" t="str">
         <x:v>S24</x:v>
       </x:c>
     </x:row>
@@ -2449,321 +2472,341 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="52" t="str">
-        <x:v>OXXO / Paynet cash voucher</x:v>
+        <x:v>Revolut Pay</x:v>
       </x:c>
       <x:c r="B5" s="53" t="str">
-        <x:v>Cash voucher</x:v>
+        <x:v>Wallet / account checkout</x:v>
       </x:c>
       <x:c r="C5" s="53" t="str">
-        <x:v>Mexico</x:v>
+        <x:v>UK/EU and Revolut-heavy markets</x:v>
       </x:c>
       <x:c r="D5" s="53" t="str">
-        <x:v>Reaches cash-preferring buyers.</x:v>
+        <x:v>Low-friction checkout for Revolut users and direct settlement into Revolut Merchant account.</x:v>
       </x:c>
       <x:c r="E5" s="53" t="str">
-        <x:v>dLocal; EBANX; Conekta; Stripe Mexico</x:v>
+        <x:v>Revolut Business Merchant Account; Revolut Gateway</x:v>
       </x:c>
       <x:c r="F5" s="54" t="str">
-        <x:v>Delayed payment; do not reserve inventory too long.</x:v>
+        <x:v>Useful UK/EU add-on, not a replacement for LatAm local rails.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="52" t="str">
-        <x:v>SPEI</x:v>
+        <x:v>OXXO / Paynet cash voucher</x:v>
       </x:c>
       <x:c r="B6" s="53" t="str">
-        <x:v>Bank transfer</x:v>
+        <x:v>Cash voucher</x:v>
       </x:c>
       <x:c r="C6" s="53" t="str">
         <x:v>Mexico</x:v>
       </x:c>
       <x:c r="D6" s="53" t="str">
-        <x:v>Important Mexican bank-transfer rail.</x:v>
+        <x:v>Reaches cash-preferring buyers.</x:v>
       </x:c>
       <x:c r="E6" s="53" t="str">
         <x:v>dLocal; EBANX; Conekta; Stripe Mexico</x:v>
       </x:c>
       <x:c r="F6" s="54" t="str">
-        <x:v>Refund and reconciliation flow matters.</x:v>
+        <x:v>Delayed payment; do not reserve inventory too long.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="52" t="str">
-        <x:v>Pix</x:v>
+        <x:v>SPEI</x:v>
       </x:c>
       <x:c r="B7" s="53" t="str">
-        <x:v>Real-time bank payment</x:v>
+        <x:v>Bank transfer</x:v>
       </x:c>
       <x:c r="C7" s="53" t="str">
-        <x:v>Brazil</x:v>
+        <x:v>Mexico</x:v>
       </x:c>
       <x:c r="D7" s="53" t="str">
-        <x:v>Brazil conversion must-have.</x:v>
+        <x:v>Important Mexican bank-transfer rail.</x:v>
       </x:c>
       <x:c r="E7" s="53" t="str">
-        <x:v>EBANX; dLocal; Mercado Pago; Stripe; Adyen</x:v>
+        <x:v>dLocal; EBANX; Conekta; Stripe Mexico</x:v>
       </x:c>
       <x:c r="F7" s="54" t="str">
-        <x:v>QR expiry and refund flow need clarity.</x:v>
+        <x:v>Refund and reconciliation flow matters.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="52" t="str">
-        <x:v>Boleto</x:v>
+        <x:v>Pix</x:v>
       </x:c>
       <x:c r="B8" s="53" t="str">
-        <x:v>Voucher</x:v>
+        <x:v>Real-time bank payment</x:v>
       </x:c>
       <x:c r="C8" s="53" t="str">
         <x:v>Brazil</x:v>
       </x:c>
       <x:c r="D8" s="53" t="str">
-        <x:v>Still useful for cash/bank voucher behavior.</x:v>
+        <x:v>Brazil conversion must-have.</x:v>
       </x:c>
       <x:c r="E8" s="53" t="str">
-        <x:v>EBANX; dLocal; Stripe Brazil</x:v>
+        <x:v>EBANX; dLocal; Mercado Pago; Stripe; Adyen</x:v>
       </x:c>
       <x:c r="F8" s="54" t="str">
-        <x:v>Delayed confirmation and inventory lock risk.</x:v>
+        <x:v>QR expiry and refund flow need clarity.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="52" t="str">
-        <x:v>Mercado Pago wallet/account money</x:v>
+        <x:v>Boleto</x:v>
       </x:c>
       <x:c r="B9" s="53" t="str">
-        <x:v>Wallet/local trust</x:v>
+        <x:v>Voucher</x:v>
       </x:c>
       <x:c r="C9" s="53" t="str">
-        <x:v>Mexico, Brazil, Argentina, Chile, Colombia</x:v>
+        <x:v>Brazil</x:v>
       </x:c>
       <x:c r="D9" s="53" t="str">
-        <x:v>Local wallet trust and installments.</x:v>
+        <x:v>Still useful for cash/bank voucher behavior.</x:v>
       </x:c>
       <x:c r="E9" s="53" t="str">
-        <x:v>Mercado Pago</x:v>
+        <x:v>EBANX; dLocal; Stripe Brazil</x:v>
       </x:c>
       <x:c r="F9" s="54" t="str">
-        <x:v>Especially relevant in Argentina and Mexico.</x:v>
+        <x:v>Delayed confirmation and inventory lock risk.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="52" t="str">
-        <x:v>PSE</x:v>
+        <x:v>Mercado Pago wallet/account money</x:v>
       </x:c>
       <x:c r="B10" s="53" t="str">
-        <x:v>Bank transfer</x:v>
+        <x:v>Wallet/local trust</x:v>
       </x:c>
       <x:c r="C10" s="53" t="str">
-        <x:v>Colombia</x:v>
+        <x:v>Mexico, Brazil, Argentina, Chile, Colombia</x:v>
       </x:c>
       <x:c r="D10" s="53" t="str">
-        <x:v>Core Colombia bank-transfer method.</x:v>
+        <x:v>Local wallet trust and installments.</x:v>
       </x:c>
       <x:c r="E10" s="53" t="str">
-        <x:v>PayU; dLocal; EBANX; Mercado Pago</x:v>
+        <x:v>Mercado Pago</x:v>
       </x:c>
       <x:c r="F10" s="54" t="str">
-        <x:v>Status sync and refunds should be tested.</x:v>
+        <x:v>Especially relevant in Argentina and Mexico.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="52" t="str">
-        <x:v>Nequi / Daviplata</x:v>
+        <x:v>PSE</x:v>
       </x:c>
       <x:c r="B11" s="53" t="str">
-        <x:v>Mobile wallet</x:v>
+        <x:v>Bank transfer</x:v>
       </x:c>
       <x:c r="C11" s="53" t="str">
         <x:v>Colombia</x:v>
       </x:c>
       <x:c r="D11" s="53" t="str">
-        <x:v>Popular mobile wallet behavior.</x:v>
+        <x:v>Core Colombia bank-transfer method.</x:v>
       </x:c>
       <x:c r="E11" s="53" t="str">
         <x:v>PayU; dLocal; EBANX; Mercado Pago</x:v>
       </x:c>
       <x:c r="F11" s="54" t="str">
-        <x:v>Requires local checkout support.</x:v>
+        <x:v>Status sync and refunds should be tested.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="52" t="str">
-        <x:v>Rapipago / Pago Facil</x:v>
+        <x:v>Nequi / Daviplata</x:v>
       </x:c>
       <x:c r="B12" s="53" t="str">
-        <x:v>Cash voucher</x:v>
+        <x:v>Mobile wallet</x:v>
       </x:c>
       <x:c r="C12" s="53" t="str">
-        <x:v>Argentina</x:v>
+        <x:v>Colombia</x:v>
       </x:c>
       <x:c r="D12" s="53" t="str">
-        <x:v>Cash/local voucher coverage.</x:v>
+        <x:v>Popular mobile wallet behavior.</x:v>
       </x:c>
       <x:c r="E12" s="53" t="str">
-        <x:v>Mercado Pago; dLocal; EBANX; PayU</x:v>
+        <x:v>PayU; dLocal; EBANX; Mercado Pago</x:v>
       </x:c>
       <x:c r="F12" s="54" t="str">
-        <x:v>Macro/FX risk dominates.</x:v>
+        <x:v>Requires local checkout support.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="52" t="str">
-        <x:v>Bizum</x:v>
+        <x:v>Rapipago / Pago Facil</x:v>
       </x:c>
       <x:c r="B13" s="53" t="str">
-        <x:v>Bank wallet</x:v>
+        <x:v>Cash voucher</x:v>
       </x:c>
       <x:c r="C13" s="53" t="str">
-        <x:v>Spain</x:v>
+        <x:v>Argentina</x:v>
       </x:c>
       <x:c r="D13" s="53" t="str">
-        <x:v>Spanish local bank-wallet habit.</x:v>
+        <x:v>Cash/local voucher coverage.</x:v>
       </x:c>
       <x:c r="E13" s="53" t="str">
-        <x:v>Local PSPs; Adyen/Stripe routes where available</x:v>
+        <x:v>Mercado Pago; dLocal; EBANX; PayU</x:v>
       </x:c>
       <x:c r="F13" s="54" t="str">
-        <x:v>Add after Spain is a serious target.</x:v>
+        <x:v>Macro/FX risk dominates.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="52" t="str">
-        <x:v>SEPA</x:v>
+        <x:v>Bizum</x:v>
       </x:c>
       <x:c r="B14" s="53" t="str">
-        <x:v>Bank transfer/direct debit</x:v>
+        <x:v>Bank wallet</x:v>
       </x:c>
       <x:c r="C14" s="53" t="str">
-        <x:v>EU</x:v>
+        <x:v>Spain</x:v>
       </x:c>
       <x:c r="D14" s="53" t="str">
-        <x:v>EU bank payment infrastructure.</x:v>
+        <x:v>Spanish local bank-wallet habit.</x:v>
       </x:c>
       <x:c r="E14" s="53" t="str">
-        <x:v>Stripe; Adyen; PayPal/Braintree</x:v>
+        <x:v>Local PSPs; Adyen/Stripe routes where available</x:v>
       </x:c>
       <x:c r="F14" s="54" t="str">
-        <x:v>Different authorization/refund timing.</x:v>
+        <x:v>Add after Spain is a serious target.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="52" t="str">
-        <x:v>Klarna / Affirm / Afterpay</x:v>
+        <x:v>SEPA</x:v>
       </x:c>
       <x:c r="B15" s="53" t="str">
-        <x:v>BNPL</x:v>
+        <x:v>Bank transfer/direct debit</x:v>
       </x:c>
       <x:c r="C15" s="53" t="str">
-        <x:v>US, UK/EU, AU/NZ</x:v>
+        <x:v>EU</x:v>
       </x:c>
       <x:c r="D15" s="53" t="str">
-        <x:v>Can improve AOV conversion.</x:v>
+        <x:v>EU bank payment infrastructure.</x:v>
       </x:c>
       <x:c r="E15" s="53" t="str">
-        <x:v>Klarna; Affirm; Afterpay; Shopify; Stripe</x:v>
+        <x:v>Stripe; Adyen; PayPal/Braintree</x:v>
       </x:c>
       <x:c r="F15" s="54" t="str">
-        <x:v>Only after margin and returns are known.</x:v>
+        <x:v>Different authorization/refund timing.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="52" t="str">
-        <x:v>Konbini</x:v>
+        <x:v>Klarna / Affirm / Afterpay</x:v>
       </x:c>
       <x:c r="B16" s="53" t="str">
-        <x:v>Convenience-store payment</x:v>
+        <x:v>BNPL</x:v>
       </x:c>
       <x:c r="C16" s="53" t="str">
-        <x:v>Japan</x:v>
+        <x:v>US, UK/EU, AU/NZ</x:v>
       </x:c>
       <x:c r="D16" s="53" t="str">
-        <x:v>Japan localized checkout expectation.</x:v>
+        <x:v>Can improve AOV conversion.</x:v>
       </x:c>
       <x:c r="E16" s="53" t="str">
-        <x:v>KOMOJU; Stripe Japan; Adyen</x:v>
+        <x:v>Klarna; Affirm; Afterpay; Shopify; Stripe</x:v>
       </x:c>
       <x:c r="F16" s="54" t="str">
-        <x:v>Delayed payment and Japanese instructions.</x:v>
+        <x:v>Only after margin and returns are known.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="52" t="str">
-        <x:v>PayPay</x:v>
+        <x:v>Konbini</x:v>
       </x:c>
       <x:c r="B17" s="53" t="str">
-        <x:v>Mobile wallet</x:v>
+        <x:v>Convenience-store payment</x:v>
       </x:c>
       <x:c r="C17" s="53" t="str">
         <x:v>Japan</x:v>
       </x:c>
       <x:c r="D17" s="53" t="str">
-        <x:v>Important Japan wallet option.</x:v>
+        <x:v>Japan localized checkout expectation.</x:v>
       </x:c>
       <x:c r="E17" s="53" t="str">
-        <x:v>KOMOJU; Adyen/local PSPs</x:v>
+        <x:v>KOMOJU; Stripe Japan; Adyen</x:v>
       </x:c>
       <x:c r="F17" s="54" t="str">
-        <x:v>Needs localized product and checkout copy.</x:v>
+        <x:v>Delayed payment and Japanese instructions.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="52" t="str">
-        <x:v>UPI</x:v>
+        <x:v>PayPay</x:v>
       </x:c>
       <x:c r="B18" s="53" t="str">
-        <x:v>Real-time bank payment</x:v>
+        <x:v>Mobile wallet</x:v>
       </x:c>
       <x:c r="C18" s="53" t="str">
-        <x:v>India</x:v>
+        <x:v>Japan</x:v>
       </x:c>
       <x:c r="D18" s="53" t="str">
-        <x:v>India online payment core.</x:v>
+        <x:v>Important Japan wallet option.</x:v>
       </x:c>
       <x:c r="E18" s="53" t="str">
-        <x:v>Razorpay; PayU India; Cashfree; PhonePe</x:v>
+        <x:v>KOMOJU; Adyen/local PSPs</x:v>
       </x:c>
       <x:c r="F18" s="54" t="str">
-        <x:v>Often requires local entity/partner.</x:v>
+        <x:v>Needs localized product and checkout copy.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="52" t="str">
+        <x:v>UPI</x:v>
+      </x:c>
+      <x:c r="B19" s="53" t="str">
+        <x:v>Real-time bank payment</x:v>
+      </x:c>
+      <x:c r="C19" s="53" t="str">
+        <x:v>India</x:v>
+      </x:c>
+      <x:c r="D19" s="53" t="str">
+        <x:v>India online payment core.</x:v>
+      </x:c>
+      <x:c r="E19" s="53" t="str">
+        <x:v>Razorpay; PayU India; Cashfree; PhonePe</x:v>
+      </x:c>
+      <x:c r="F19" s="54" t="str">
+        <x:v>Often requires local entity/partner.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="52" t="str">
         <x:v>Interac</x:v>
       </x:c>
-      <x:c r="B19" s="53" t="str">
+      <x:c r="B20" s="53" t="str">
         <x:v>Debit/transfer</x:v>
       </x:c>
-      <x:c r="C19" s="53" t="str">
+      <x:c r="C20" s="53" t="str">
         <x:v>Canada</x:v>
       </x:c>
-      <x:c r="D19" s="53" t="str">
+      <x:c r="D20" s="53" t="str">
         <x:v>Local Canadian payment behavior.</x:v>
       </x:c>
-      <x:c r="E19" s="53" t="str">
+      <x:c r="E20" s="53" t="str">
         <x:v>Stripe/Adyen/local processors depending setup</x:v>
       </x:c>
-      <x:c r="F19" s="54" t="str">
+      <x:c r="F20" s="54" t="str">
         <x:v>Useful for CAD-localized checkout.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="63" t="str">
+    <x:row r="21">
+      <x:c r="A21" s="63" t="str">
         <x:v>COD</x:v>
       </x:c>
-      <x:c r="B20" s="64" t="str">
+      <x:c r="B21" s="64" t="str">
         <x:v>Cash on delivery</x:v>
       </x:c>
-      <x:c r="C20" s="64" t="str">
+      <x:c r="C21" s="64" t="str">
         <x:v>India, Colombia, Japan in some contexts</x:v>
       </x:c>
-      <x:c r="D20" s="64" t="str">
+      <x:c r="D21" s="64" t="str">
         <x:v>Trust booster in lower-card-trust markets.</x:v>
       </x:c>
-      <x:c r="E20" s="64" t="str">
+      <x:c r="E21" s="64" t="str">
         <x:v>Local logistics/marketplace</x:v>
       </x:c>
-      <x:c r="F20" s="65" t="str">
+      <x:c r="F21" s="65" t="str">
         <x:v>High refusal and return risk; avoid for first DTC tests.</x:v>
       </x:c>
     </x:row>
@@ -2857,7 +2900,7 @@
         <x:v>Seller payout stack</x:v>
       </x:c>
       <x:c r="B6" s="53" t="str">
-        <x:v>Airwallex + Payoneer/WorldFirst/PingPong backup</x:v>
+        <x:v>Airwallex/Revolut + Payoneer/WorldFirst/PingPong backup</x:v>
       </x:c>
       <x:c r="C6" s="53" t="str">
         <x:v>Multiple platforms and currencies</x:v>
@@ -2868,57 +2911,71 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="52" t="str">
-        <x:v>Supplier payments</x:v>
+        <x:v>UK/EU business account + checkout backup</x:v>
       </x:c>
       <x:c r="B7" s="53" t="str">
-        <x:v>WorldFirst / Airwallex / Wise / LianLian / PingPong</x:v>
+        <x:v>Revolut Business + Stripe/Shopify + PayPal</x:v>
       </x:c>
       <x:c r="C7" s="53" t="str">
-        <x:v>Paying Chinese suppliers from overseas sales</x:v>
+        <x:v>UK/EU/AU entity wants FX plus payment acceptance in one account</x:v>
       </x:c>
       <x:c r="D7" s="54" t="str">
-        <x:v>Compare FX spread, transfer limits, and supplier acceptance.</x:v>
+        <x:v>Treat Revolut as add-on/secondary PSP until payment volume and risk controls are proven.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="52" t="str">
-        <x:v>EU launch</x:v>
+        <x:v>Supplier payments</x:v>
       </x:c>
       <x:c r="B8" s="53" t="str">
-        <x:v>Stripe/Shopify + PayPal + Klarna/SEPA + IOSS/VAT process</x:v>
+        <x:v>WorldFirst / Airwallex / Wise / LianLian / PingPong</x:v>
       </x:c>
       <x:c r="C8" s="53" t="str">
-        <x:v>Spain/Germany/EU expansion</x:v>
+        <x:v>Paying Chinese suppliers from overseas sales</x:v>
       </x:c>
       <x:c r="D8" s="54" t="str">
-        <x:v>Compliance and returns matter more than adding every payment method.</x:v>
+        <x:v>Compare FX spread, transfer limits, and supplier acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="52" t="str">
+        <x:v>EU launch</x:v>
+      </x:c>
+      <x:c r="B9" s="53" t="str">
+        <x:v>Stripe/Shopify + PayPal + Klarna/SEPA + IOSS/VAT process</x:v>
+      </x:c>
+      <x:c r="C9" s="53" t="str">
+        <x:v>Spain/Germany/EU expansion</x:v>
+      </x:c>
+      <x:c r="D9" s="54" t="str">
+        <x:v>Compliance and returns matter more than adding every payment method.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="52" t="str">
         <x:v>Japan launch</x:v>
       </x:c>
-      <x:c r="B9" s="53" t="str">
+      <x:c r="B10" s="53" t="str">
         <x:v>KOMOJU or Stripe Japan + cards + Konbini + PayPay</x:v>
       </x:c>
-      <x:c r="C9" s="53" t="str">
+      <x:c r="C10" s="53" t="str">
         <x:v>Japan-specific product-market fit</x:v>
       </x:c>
-      <x:c r="D9" s="54" t="str">
+      <x:c r="D10" s="54" t="str">
         <x:v>No Japan payment stack can rescue poor localization.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="63" t="str">
+    <x:row r="11">
+      <x:c r="A11" s="63" t="str">
         <x:v>India launch</x:v>
       </x:c>
-      <x:c r="B10" s="64" t="str">
+      <x:c r="B11" s="64" t="str">
         <x:v>Local PSP such as Razorpay/PayU/Cashfree + UPI</x:v>
       </x:c>
-      <x:c r="C10" s="64" t="str">
+      <x:c r="C11" s="64" t="str">
         <x:v>Only with local partner/entity</x:v>
       </x:c>
-      <x:c r="D10" s="65" t="str">
+      <x:c r="D11" s="65" t="str">
         <x:v>COD and logistics must be operationally modeled first.</x:v>
       </x:c>
     </x:row>
@@ -3344,17 +3401,73 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="63" t="str">
+      <x:c r="A30" s="52" t="str">
         <x:v>S30</x:v>
       </x:c>
-      <x:c r="B30" s="64" t="str">
+      <x:c r="B30" s="53" t="str">
         <x:v>Trade.gov Australia ecommerce</x:v>
       </x:c>
-      <x:c r="C30" s="64" t="str">
+      <x:c r="C30" s="53" t="str">
         <x:v>Australia ecommerce context.</x:v>
       </x:c>
-      <x:c r="D30" s="65" t="str">
+      <x:c r="D30" s="54" t="str">
         <x:v>https://www.trade.gov/country-commercial-guides/australia-ecommerce</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="52" t="str">
+        <x:v>S31</x:v>
+      </x:c>
+      <x:c r="B31" s="53" t="str">
+        <x:v>Revolut Business multi-currency accounts</x:v>
+      </x:c>
+      <x:c r="C31" s="53" t="str">
+        <x:v>Multi-currency business account, FX, supplier/customer payment context.</x:v>
+      </x:c>
+      <x:c r="D31" s="54" t="str">
+        <x:v>https://www.revolut.com/business/multi-currency-accounts/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="52" t="str">
+        <x:v>S32</x:v>
+      </x:c>
+      <x:c r="B32" s="53" t="str">
+        <x:v>Revolut Business accept payments</x:v>
+      </x:c>
+      <x:c r="C32" s="53" t="str">
+        <x:v>Merchant account, payment gateway, settlement, and Revolut Pay context.</x:v>
+      </x:c>
+      <x:c r="D32" s="54" t="str">
+        <x:v>https://www.revolut.com/business/accept-payments/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="52" t="str">
+        <x:v>S33</x:v>
+      </x:c>
+      <x:c r="B33" s="53" t="str">
+        <x:v>Revolut Merchant API</x:v>
+      </x:c>
+      <x:c r="C33" s="53" t="str">
+        <x:v>Online payment methods, widgets, hosted checkout, and plugins.</x:v>
+      </x:c>
+      <x:c r="D33" s="54" t="str">
+        <x:v>https://developer.revolut.com/docs/accept-payments/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="63" t="str">
+        <x:v>S34</x:v>
+      </x:c>
+      <x:c r="B34" s="64" t="str">
+        <x:v>Revolut merchant eligibility</x:v>
+      </x:c>
+      <x:c r="C34" s="64" t="str">
+        <x:v>Supported merchant account countries and eligibility constraints.</x:v>
+      </x:c>
+      <x:c r="D34" s="65" t="str">
+        <x:v>https://help.revolut.com/help/merchant-accounts/setting-up-a-merchant-account/who-can-apply-for-a-merchant-account/business/</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>